<commit_message>
add email for all usecases , and fixed UI typos like Book999
</commit_message>
<xml_diff>
--- a/COEP_VenuesInfo.xlsx
+++ b/COEP_VenuesInfo.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="27">
   <si>
     <t>venue_name</t>
   </si>
@@ -32,15 +32,6 @@
   </si>
   <si>
     <t>Academic Complex</t>
-  </si>
-  <si>
-    <t>North Campus, Beside COEP Boat Club</t>
-  </si>
-  <si>
-    <t>800</t>
-  </si>
-  <si>
-    <t>Projector, Screen,Wifi</t>
   </si>
   <si>
     <r>
@@ -50,17 +41,17 @@
         <color indexed="11"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>ac.test@gmail.com</t>
+      <t>https://lh3.googleusercontent.com/p/AF1QipNdWaJtM7bFBSsRiZP7Pk-aJiFde2ObOTTm81vT=s680-w680-h510</t>
     </r>
   </si>
   <si>
-    <t>FOSS</t>
-  </si>
-  <si>
-    <t>North Campus, Third Floor,Electronics Extension(New) Building,</t>
-  </si>
-  <si>
-    <t>PCs, Projector, AC, Wifi</t>
+    <t>North Campus, Beside COEP Boat Club</t>
+  </si>
+  <si>
+    <t>800</t>
+  </si>
+  <si>
+    <t>Projector, Screen,Wifi</t>
   </si>
   <si>
     <r>
@@ -70,17 +61,11 @@
         <color indexed="11"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>foss.test@gmail.com</t>
+      <t>arnav.davpune@gmail.com</t>
     </r>
   </si>
   <si>
-    <t>BHAU</t>
-  </si>
-  <si>
-    <t>Ground floor, Bhau Institute, COEP Technological University</t>
-  </si>
-  <si>
-    <t>AC,Projector,Sound Systems, Wifi</t>
+    <t>FOSS</t>
   </si>
   <si>
     <r>
@@ -90,17 +75,17 @@
         <color indexed="11"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>bhau.test@gmail.com</t>
+      <t>https://foss.coep.org.in/cofsug/services/foss-lab.png</t>
     </r>
   </si>
   <si>
+    <t>North Campus, Third Floor,Electronics Extension(New) Building,</t>
+  </si>
+  <si>
+    <t>PCs, Projector, AC, Wifi</t>
+  </si>
+  <si>
     <t>Cognizant Lab</t>
-  </si>
-  <si>
-    <t>Ground Floor Academic Complex, North Campus</t>
-  </si>
-  <si>
-    <t>AC,Projector,Sound Systems, Wifi,PCs</t>
   </si>
   <si>
     <r>
@@ -110,8 +95,51 @@
         <color indexed="11"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>cognizant.test@gmail.com</t>
+      <t>https://www.campustimespune.com/wp-content/uploads/2016/10/Cognizant-Lab-Campus-Images-Pune.jpg</t>
     </r>
+  </si>
+  <si>
+    <t>Ground Floor Academic Complex, North Campus</t>
+  </si>
+  <si>
+    <t>AC,Projector,Sound Systems, Wifi,PCs</t>
+  </si>
+  <si>
+    <t>Main Auditorium</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color indexed="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>https://upload.wikimedia.org/wikipedia/commons/thumb/c/ca/College_of_Engineering%2C_Pune_Auditorium_%28Stage_View%29.jpg/800px-College_of_Engineering%2C_Pune_Auditorium_%28Stage_View%29.jpg?20111223052524</t>
+    </r>
+  </si>
+  <si>
+    <t>South Campus , near library</t>
+  </si>
+  <si>
+    <t>AC,Projector,Sound Systems, Wifi</t>
+  </si>
+  <si>
+    <t>Mini Auditorium</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color indexed="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>https://www.campustimespune.com/wp-content/uploads/2015/10/COEP-mindspark-workshop.jpg</t>
+    </r>
+  </si>
+  <si>
+    <t>North Campus, near Academic Complex</t>
   </si>
 </sst>
 </file>
@@ -143,12 +171,12 @@
       <name val="Times New Roman"/>
     </font>
     <font>
+      <u val="single"/>
       <sz val="11"/>
       <color indexed="11"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <u val="single"/>
       <sz val="11"/>
       <color indexed="11"/>
       <name val="Calibri"/>
@@ -320,10 +348,10 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -367,191 +395,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>353520</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>21959</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2379960</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>1201320</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 5" descr="Picture 5"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1">
-          <a:extLst/>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1610819" y="204839"/>
-          <a:ext cx="2026442" cy="1179361"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
-        </a:ln>
-        <a:effectLst/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>379079</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>33120</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2450520</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>1289519</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 7" descr="Picture 7"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2">
-          <a:extLst/>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1636379" y="2982060"/>
-          <a:ext cx="2071442" cy="1256400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
-        </a:ln>
-        <a:effectLst/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>298799</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>40680</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2408760</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>1289520</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 8" descr="Picture 8"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId3">
-          <a:extLst/>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1556099" y="4315500"/>
-          <a:ext cx="2109961" cy="1248841"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
-        </a:ln>
-        <a:effectLst/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>124919</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>19080</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2722680</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>1491479</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 9" descr="Picture 9"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId4">
-          <a:extLst/>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1382219" y="1428780"/>
-          <a:ext cx="2597762" cy="1472400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
-        </a:ln>
-        <a:effectLst/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -747,9 +590,12 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1023,9 +869,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1574,11 +1423,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="14.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="16.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="40.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="99.7578" style="1" customWidth="1"/>
     <col min="3" max="3" width="53.1719" style="1" customWidth="1"/>
     <col min="4" max="4" width="20" style="1" customWidth="1"/>
     <col min="5" max="5" width="48.8516" style="1" customWidth="1"/>
@@ -1610,126 +1459,143 @@
       <c r="A2" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="B2" s="7"/>
+      <c r="B2" t="s" s="5">
+        <v>7</v>
+      </c>
       <c r="C2" t="s" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s" s="5">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s" s="8">
         <v>10</v>
+      </c>
+      <c r="F2" t="s" s="7">
+        <v>11</v>
       </c>
     </row>
     <row r="3" ht="121.2" customHeight="1">
       <c r="A3" t="s" s="5">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s" s="5">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s" s="5">
+        <v>14</v>
+      </c>
+      <c r="D3" s="8">
+        <v>40</v>
+      </c>
+      <c r="E3" t="s" s="5">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s" s="7">
         <v>11</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" t="s" s="5">
-        <v>12</v>
-      </c>
-      <c r="D3" s="7">
-        <v>40</v>
-      </c>
-      <c r="E3" t="s" s="5">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s" s="8">
-        <v>14</v>
-      </c>
     </row>
-    <row r="4" ht="104.4" customHeight="1">
+    <row r="4" ht="108" customHeight="1">
       <c r="A4" t="s" s="5">
-        <v>15</v>
-      </c>
-      <c r="B4" s="7"/>
+        <v>16</v>
+      </c>
+      <c r="B4" t="s" s="5">
+        <v>17</v>
+      </c>
       <c r="C4" t="s" s="5">
-        <v>16</v>
-      </c>
-      <c r="D4" s="7">
-        <v>120</v>
+        <v>18</v>
+      </c>
+      <c r="D4" s="8">
+        <v>200</v>
       </c>
       <c r="E4" t="s" s="5">
-        <v>17</v>
-      </c>
-      <c r="F4" t="s" s="8">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="F4" t="s" s="7">
+        <v>11</v>
       </c>
     </row>
-    <row r="5" ht="108" customHeight="1">
+    <row r="5" ht="14.4" customHeight="1">
       <c r="A5" t="s" s="5">
-        <v>19</v>
-      </c>
-      <c r="B5" s="7"/>
+        <v>20</v>
+      </c>
+      <c r="B5" t="s" s="5">
+        <v>21</v>
+      </c>
       <c r="C5" t="s" s="5">
-        <v>20</v>
-      </c>
-      <c r="D5" s="7">
-        <v>200</v>
+        <v>22</v>
+      </c>
+      <c r="D5" s="8">
+        <v>100</v>
       </c>
       <c r="E5" t="s" s="5">
-        <v>21</v>
-      </c>
-      <c r="F5" t="s" s="8">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="F5" t="s" s="7">
+        <v>11</v>
       </c>
     </row>
     <row r="6" ht="14.4" customHeight="1">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
+      <c r="A6" t="s" s="5">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s" s="5">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s" s="5">
+        <v>26</v>
+      </c>
+      <c r="D6" s="8">
+        <v>180</v>
+      </c>
+      <c r="E6" t="s" s="5">
+        <v>23</v>
+      </c>
+      <c r="F6" t="s" s="7">
+        <v>11</v>
+      </c>
     </row>
     <row r="7" ht="14.4" customHeight="1">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
     </row>
     <row r="8" ht="14.4" customHeight="1">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="11"/>
     </row>
     <row r="9" ht="14.4" customHeight="1">
-      <c r="A9" s="9"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="11"/>
-    </row>
-    <row r="10" ht="14.4" customHeight="1">
-      <c r="A10" s="12"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="14"/>
+      <c r="A9" s="12"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="14"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" location="" tooltip="" display="ac.test@gmail.com"/>
-    <hyperlink ref="F3" r:id="rId2" location="" tooltip="" display="foss.test@gmail.com"/>
-    <hyperlink ref="F4" r:id="rId3" location="" tooltip="" display="bhau.test@gmail.com"/>
-    <hyperlink ref="F5" r:id="rId4" location="" tooltip="" display="cognizant.test@gmail.com"/>
+    <hyperlink ref="B2" r:id="rId1" location="" tooltip="" display="https://lh3.googleusercontent.com/p/AF1QipNdWaJtM7bFBSsRiZP7Pk-aJiFde2ObOTTm81vT=s680-w680-h510"/>
+    <hyperlink ref="F2" r:id="rId2" location="" tooltip="" display="arnav.davpune@gmail.com"/>
+    <hyperlink ref="B3" r:id="rId3" location="" tooltip="" display="https://foss.coep.org.in/cofsug/services/foss-lab.png"/>
+    <hyperlink ref="F3" r:id="rId4" location="" tooltip="" display="arnav.davpune@gmail.com"/>
+    <hyperlink ref="B4" r:id="rId5" location="" tooltip="" display="https://www.campustimespune.com/wp-content/uploads/2016/10/Cognizant-Lab-Campus-Images-Pune.jpg"/>
+    <hyperlink ref="F4" r:id="rId6" location="" tooltip="" display="arnav.davpune@gmail.com"/>
+    <hyperlink ref="B5" r:id="rId7" location="" tooltip="" display="https://upload.wikimedia.org/wikipedia/commons/thumb/c/ca/College_of_Engineering%2C_Pune_Auditorium_%28Stage_View%29.jpg/800px-College_of_Engineering%2C_Pune_Auditorium_%28Stage_View%29.jpg?20111223052524"/>
+    <hyperlink ref="F5" r:id="rId8" location="" tooltip="" display="arnav.davpune@gmail.com"/>
+    <hyperlink ref="B6" r:id="rId9" location="" tooltip="" display="https://www.campustimespune.com/wp-content/uploads/2015/10/COEP-mindspark-workshop.jpg"/>
+    <hyperlink ref="F6" r:id="rId10" location="" tooltip="" display="arnav.davpune@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811" footer="0.3"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
-  <drawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>